<commit_message>
add new part 6
</commit_message>
<xml_diff>
--- a/public/flashcard_template.xlsx
+++ b/public/flashcard_template.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D70F0531-3B12-4FB6-B097-DC7785B9EADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4E76473-2429-46E1-BAA0-3C0ABCB6FD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Buổi 2" sheetId="1" r:id="rId1"/>
     <sheet name="Buổi 3" sheetId="2" r:id="rId2"/>
     <sheet name="Buổi 4" sheetId="3" r:id="rId3"/>
     <sheet name="Buổi 5" sheetId="5" r:id="rId4"/>
+    <sheet name="Buổi 6" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1020" uniqueCount="890">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1275" uniqueCount="1140">
   <si>
     <t>English</t>
   </si>
@@ -2688,6 +2689,756 @@
   </si>
   <si>
     <t>basket</t>
+  </si>
+  <si>
+    <t>/ˈtredmɪl/</t>
+  </si>
+  <si>
+    <t>máy chạy bộ</t>
+  </si>
+  <si>
+    <t>He is running on the treadmill.</t>
+  </si>
+  <si>
+    <t>Anh ấy đang chạy trên máy chạy bộ.</t>
+  </si>
+  <si>
+    <t>/ˈbɑːtl/</t>
+  </si>
+  <si>
+    <t>chai</t>
+  </si>
+  <si>
+    <t>There is a bottle on the table.</t>
+  </si>
+  <si>
+    <t>Có một cái chai trên bàn.</t>
+  </si>
+  <si>
+    <t>/boʊl/</t>
+  </si>
+  <si>
+    <t>cái bát</t>
+  </si>
+  <si>
+    <t>She is holding a bowl.</t>
+  </si>
+  <si>
+    <t>Cô ấy đang cầm một cái bát.</t>
+  </si>
+  <si>
+    <t>/ˈmenjuː/</t>
+  </si>
+  <si>
+    <t>thực đơn</t>
+  </si>
+  <si>
+    <t>The waiter handed us the menu.</t>
+  </si>
+  <si>
+    <t>Người phục vụ đưa cho chúng tôi thực đơn.</t>
+  </si>
+  <si>
+    <t>/ˈteɪblklɔːθ/</t>
+  </si>
+  <si>
+    <t>khăn trải bàn</t>
+  </si>
+  <si>
+    <t>The tablecloth is white.</t>
+  </si>
+  <si>
+    <t>Khăn trải bàn màu trắng.</t>
+  </si>
+  <si>
+    <t>/ˈeriə/</t>
+  </si>
+  <si>
+    <t>khu vực</t>
+  </si>
+  <si>
+    <t>This area is very quiet.</t>
+  </si>
+  <si>
+    <t>Khu vực này rất yên tĩnh.</t>
+  </si>
+  <si>
+    <t>/miːl/</t>
+  </si>
+  <si>
+    <t>bữa ăn</t>
+  </si>
+  <si>
+    <t>They are enjoying a meal.</t>
+  </si>
+  <si>
+    <t>Họ đang thưởng thức một bữa ăn.</t>
+  </si>
+  <si>
+    <t>/pleɪt/</t>
+  </si>
+  <si>
+    <t>cái đĩa</t>
+  </si>
+  <si>
+    <t>The food is on the plate.</t>
+  </si>
+  <si>
+    <t>Thức ăn ở trên đĩa.</t>
+  </si>
+  <si>
+    <t>/ʌmˈbrelə/</t>
+  </si>
+  <si>
+    <t>cái ô</t>
+  </si>
+  <si>
+    <t>She is carrying an umbrella.</t>
+  </si>
+  <si>
+    <t>Cô ấy đang cầm ô.</t>
+  </si>
+  <si>
+    <t>/ˈkaʊntər/</t>
+  </si>
+  <si>
+    <t>cái quầy</t>
+  </si>
+  <si>
+    <t>He is standing at the counter.</t>
+  </si>
+  <si>
+    <t>Anh ấy đang đứng ở quầy.</t>
+  </si>
+  <si>
+    <t>/lɔːn/</t>
+  </si>
+  <si>
+    <t>bãi cỏ</t>
+  </si>
+  <si>
+    <t>The lawn is freshly cut.</t>
+  </si>
+  <si>
+    <t>Bãi cỏ vừa được cắt.</t>
+  </si>
+  <si>
+    <t>/pərˈfɔːrməns/</t>
+  </si>
+  <si>
+    <t>buổi biểu diễn</t>
+  </si>
+  <si>
+    <t>The performance was excellent.</t>
+  </si>
+  <si>
+    <t>Buổi biểu diễn rất tuyệt vời.</t>
+  </si>
+  <si>
+    <t>/taɪl/</t>
+  </si>
+  <si>
+    <t>gạch lát</t>
+  </si>
+  <si>
+    <t>The floor is covered with tiles.</t>
+  </si>
+  <si>
+    <t>Sàn nhà được lát gạch.</t>
+  </si>
+  <si>
+    <t>/saɪn/</t>
+  </si>
+  <si>
+    <t>biển báo</t>
+  </si>
+  <si>
+    <t>There is a sign near the road.</t>
+  </si>
+  <si>
+    <t>Có một biển báo gần con đường.</t>
+  </si>
+  <si>
+    <t>/ˈpʌdl/</t>
+  </si>
+  <si>
+    <t>vũng nước</t>
+  </si>
+  <si>
+    <t>A puddle is on the pavement.</t>
+  </si>
+  <si>
+    <t>Có một vũng nước trên vỉa hè.</t>
+  </si>
+  <si>
+    <t>/ˈpeɪvmənt/</t>
+  </si>
+  <si>
+    <t>vỉa hè</t>
+  </si>
+  <si>
+    <t>People are walking on the pavement.</t>
+  </si>
+  <si>
+    <t>Mọi người đang đi trên vỉa hè.</t>
+  </si>
+  <si>
+    <t>/kənˈstrʌkʃən ˈwɜːrkər/</t>
+  </si>
+  <si>
+    <t>công nhân xây dựng</t>
+  </si>
+  <si>
+    <t>The construction worker is wearing a hard hat.</t>
+  </si>
+  <si>
+    <t>Người công nhân xây dựng đang đội mũ bảo hộ.</t>
+  </si>
+  <si>
+    <t>/ˈentrəns/</t>
+  </si>
+  <si>
+    <t>lối vào</t>
+  </si>
+  <si>
+    <t>The entrance is crowded.</t>
+  </si>
+  <si>
+    <t>Lối vào rất đông.</t>
+  </si>
+  <si>
+    <t>/ˈkʌbərd/</t>
+  </si>
+  <si>
+    <t>tủ đựng đồ</t>
+  </si>
+  <si>
+    <t>The plates are in the cupboard.</t>
+  </si>
+  <si>
+    <t>Những chiếc đĩa ở trong tủ.</t>
+  </si>
+  <si>
+    <t>/juːˈtensl/</t>
+  </si>
+  <si>
+    <t>dụng cụ nhà bếp</t>
+  </si>
+  <si>
+    <t>She is washing a utensil.</t>
+  </si>
+  <si>
+    <t>Cô ấy đang rửa một dụng cụ nhà bếp.</t>
+  </si>
+  <si>
+    <t>/ˈaʊtlet/</t>
+  </si>
+  <si>
+    <t>ổ điện</t>
+  </si>
+  <si>
+    <t>The charger is plugged into the outlet.</t>
+  </si>
+  <si>
+    <t>Bộ sạc được cắm vào ổ điện.</t>
+  </si>
+  <si>
+    <t>/læmp/</t>
+  </si>
+  <si>
+    <t>đèn</t>
+  </si>
+  <si>
+    <t>The lamp is on the desk.</t>
+  </si>
+  <si>
+    <t>Chiếc đèn ở trên bàn.</t>
+  </si>
+  <si>
+    <t>/freɪm/</t>
+  </si>
+  <si>
+    <t>khung</t>
+  </si>
+  <si>
+    <t>The picture is in a frame.</t>
+  </si>
+  <si>
+    <t>Bức tranh ở trong khung.</t>
+  </si>
+  <si>
+    <t>/ˈlædər/</t>
+  </si>
+  <si>
+    <t>cái thang</t>
+  </si>
+  <si>
+    <t>He is standing on a ladder.</t>
+  </si>
+  <si>
+    <t>Anh ấy đang đứng trên thang.</t>
+  </si>
+  <si>
+    <t>/ˈpʌzl/</t>
+  </si>
+  <si>
+    <t>câu đố/ trò xếp hình</t>
+  </si>
+  <si>
+    <t>The child is doing a puzzle.</t>
+  </si>
+  <si>
+    <t>Đứa trẻ đang chơi trò xếp hình.</t>
+  </si>
+  <si>
+    <t>/ˈswetər/</t>
+  </si>
+  <si>
+    <t>áo len</t>
+  </si>
+  <si>
+    <t>She is wearing a sweater.</t>
+  </si>
+  <si>
+    <t>Cô ấy đang mặc áo len.</t>
+  </si>
+  <si>
+    <t>/ˈɡlæsɪz/</t>
+  </si>
+  <si>
+    <t>kính mắt</t>
+  </si>
+  <si>
+    <t>He is wearing glasses.</t>
+  </si>
+  <si>
+    <t>Anh ấy đang đeo kính.</t>
+  </si>
+  <si>
+    <t>/ˈhæmər/</t>
+  </si>
+  <si>
+    <t>cái búa</t>
+  </si>
+  <si>
+    <t>The hammer is on the floor.</t>
+  </si>
+  <si>
+    <t>Cái búa ở trên sàn.</t>
+  </si>
+  <si>
+    <t>/ɡeɪt/</t>
+  </si>
+  <si>
+    <t>cổng</t>
+  </si>
+  <si>
+    <t>The gate is open.</t>
+  </si>
+  <si>
+    <t>Cánh cổng đang mở.</t>
+  </si>
+  <si>
+    <t>/ˈreɪlɪŋ/</t>
+  </si>
+  <si>
+    <t>lan can</t>
+  </si>
+  <si>
+    <t>She is holding the railing.</t>
+  </si>
+  <si>
+    <t>Cô ấy đang vịn lan can.</t>
+  </si>
+  <si>
+    <t>/ˈkɑːləm/</t>
+  </si>
+  <si>
+    <t>cột</t>
+  </si>
+  <si>
+    <t>The building has tall columns.</t>
+  </si>
+  <si>
+    <t>Tòa nhà có những chiếc cột cao.</t>
+  </si>
+  <si>
+    <t>/ˈsɜːrvər/</t>
+  </si>
+  <si>
+    <t>người phục vụ</t>
+  </si>
+  <si>
+    <t>The server is carrying plates.</t>
+  </si>
+  <si>
+    <t>Người phục vụ đang bưng đĩa.</t>
+  </si>
+  <si>
+    <t>/ˈkeɪbl/</t>
+  </si>
+  <si>
+    <t>dây cáp</t>
+  </si>
+  <si>
+    <t>The cable is under the desk.</t>
+  </si>
+  <si>
+    <t>Dây cáp ở dưới bàn.</t>
+  </si>
+  <si>
+    <t>/stuːl/</t>
+  </si>
+  <si>
+    <t>ghế đẩu</t>
+  </si>
+  <si>
+    <t>He is sitting on a stool.</t>
+  </si>
+  <si>
+    <t>Anh ấy đang ngồi trên ghế đẩu.</t>
+  </si>
+  <si>
+    <t>/ˈkæbɪnət/</t>
+  </si>
+  <si>
+    <t>tủ</t>
+  </si>
+  <si>
+    <t>The cabinet is made of wood.</t>
+  </si>
+  <si>
+    <t>Chiếc tủ được làm bằng gỗ.</t>
+  </si>
+  <si>
+    <t>/ˈskæfoʊld/</t>
+  </si>
+  <si>
+    <t>giàn giáo</t>
+  </si>
+  <si>
+    <t>Workers are standing on the scaffold.</t>
+  </si>
+  <si>
+    <t>Công nhân đang đứng trên giàn giáo.</t>
+  </si>
+  <si>
+    <t>/ˈmɑːrkɪt stænd/</t>
+  </si>
+  <si>
+    <t>quầy hàng ở chợ</t>
+  </si>
+  <si>
+    <t>The fruit is displayed on the market stand.</t>
+  </si>
+  <si>
+    <t>Trái cây được bày trên quầy hàng.</t>
+  </si>
+  <si>
+    <t>/ˈpɪlər/</t>
+  </si>
+  <si>
+    <t>trụ cột</t>
+  </si>
+  <si>
+    <t>The roof is supported by pillars.</t>
+  </si>
+  <si>
+    <t>Mái nhà được chống đỡ bởi các trụ cột.</t>
+  </si>
+  <si>
+    <t>/ˈpoʊdiəm/</t>
+  </si>
+  <si>
+    <t>bục phát biểu</t>
+  </si>
+  <si>
+    <t>The speaker is standing at the podium.</t>
+  </si>
+  <si>
+    <t>Diễn giả đang đứng ở bục phát biểu.</t>
+  </si>
+  <si>
+    <t>/pɪr/</t>
+  </si>
+  <si>
+    <t>bến tàu/ cầu tàu</t>
+  </si>
+  <si>
+    <t>People are walking on the pier.</t>
+  </si>
+  <si>
+    <t>Mọi người đang đi trên cầu tàu.</t>
+  </si>
+  <si>
+    <t>/kreɪt/</t>
+  </si>
+  <si>
+    <t>thùng gỗ / sọt</t>
+  </si>
+  <si>
+    <t>The apples are in a crate.</t>
+  </si>
+  <si>
+    <t>Những quả táo ở trong thùng.</t>
+  </si>
+  <si>
+    <t>/ˈstɪrɪŋ wiːl/</t>
+  </si>
+  <si>
+    <t>vô lăng</t>
+  </si>
+  <si>
+    <t>He is holding the steering wheel.</t>
+  </si>
+  <si>
+    <t>Anh ấy đang cầm vô lăng.</t>
+  </si>
+  <si>
+    <t>/ˈpætioʊ/</t>
+  </si>
+  <si>
+    <t>sân hiên</t>
+  </si>
+  <si>
+    <t>They are sitting on the patio.</t>
+  </si>
+  <si>
+    <t>Họ đang ngồi ở sân hiên.</t>
+  </si>
+  <si>
+    <t>/kɜːrb/</t>
+  </si>
+  <si>
+    <t>lề đường</t>
+  </si>
+  <si>
+    <t>The car is parked by the curb.</t>
+  </si>
+  <si>
+    <t>Chiếc xe được đậu bên lề đường.</t>
+  </si>
+  <si>
+    <t>/ræmp/</t>
+  </si>
+  <si>
+    <t>đường dốc</t>
+  </si>
+  <si>
+    <t>The wheelchair is on the ramp.</t>
+  </si>
+  <si>
+    <t>Chiếc xe lăn đang ở trên đường dốc.</t>
+  </si>
+  <si>
+    <t>/ˈwɪndoʊ ledʒ/</t>
+  </si>
+  <si>
+    <t>bệ cửa sổ</t>
+  </si>
+  <si>
+    <t>A plant is on the window ledge.</t>
+  </si>
+  <si>
+    <t>Một chậu cây ở trên bệ cửa sổ.</t>
+  </si>
+  <si>
+    <t>/ˈʃædoʊ/</t>
+  </si>
+  <si>
+    <t>bóng / bóng râm</t>
+  </si>
+  <si>
+    <t>The tree casts a shadow.</t>
+  </si>
+  <si>
+    <t>Cái cây tạo ra bóng râm.</t>
+  </si>
+  <si>
+    <t>/ˈpærəlel/</t>
+  </si>
+  <si>
+    <t>song song</t>
+  </si>
+  <si>
+    <t>The lines are parallel.</t>
+  </si>
+  <si>
+    <t>Các đường thẳng song song.</t>
+  </si>
+  <si>
+    <t>/ˈlæmpˌpoʊst/</t>
+  </si>
+  <si>
+    <t>cột đèn</t>
+  </si>
+  <si>
+    <t>The lamppost is near the road.</t>
+  </si>
+  <si>
+    <t>Cột đèn ở gần con đường.</t>
+  </si>
+  <si>
+    <t>/ˈkɔːrɪdɔːr/</t>
+  </si>
+  <si>
+    <t>hành lang</t>
+  </si>
+  <si>
+    <t>She is walking down the corridor.</t>
+  </si>
+  <si>
+    <t>Cô ấy đang đi dọc hành lang.</t>
+  </si>
+  <si>
+    <t>treadmill</t>
+  </si>
+  <si>
+    <t>bottle</t>
+  </si>
+  <si>
+    <t>bowl</t>
+  </si>
+  <si>
+    <t>menu</t>
+  </si>
+  <si>
+    <t>tablecloth</t>
+  </si>
+  <si>
+    <t>area</t>
+  </si>
+  <si>
+    <t>meal</t>
+  </si>
+  <si>
+    <t>plate</t>
+  </si>
+  <si>
+    <t>umbrella</t>
+  </si>
+  <si>
+    <t>counter</t>
+  </si>
+  <si>
+    <t>lawn</t>
+  </si>
+  <si>
+    <t>performance</t>
+  </si>
+  <si>
+    <t>tile</t>
+  </si>
+  <si>
+    <t>sign</t>
+  </si>
+  <si>
+    <t>puddle</t>
+  </si>
+  <si>
+    <t>pavement</t>
+  </si>
+  <si>
+    <t>construction worker</t>
+  </si>
+  <si>
+    <t>entrance</t>
+  </si>
+  <si>
+    <t>cupboard</t>
+  </si>
+  <si>
+    <t>utensil</t>
+  </si>
+  <si>
+    <t>outlet</t>
+  </si>
+  <si>
+    <t>lamp</t>
+  </si>
+  <si>
+    <t>frame</t>
+  </si>
+  <si>
+    <t>ladder</t>
+  </si>
+  <si>
+    <t>puzzle</t>
+  </si>
+  <si>
+    <t>sweater</t>
+  </si>
+  <si>
+    <t>glasses</t>
+  </si>
+  <si>
+    <t>hammer</t>
+  </si>
+  <si>
+    <t>gate</t>
+  </si>
+  <si>
+    <t>railing</t>
+  </si>
+  <si>
+    <t>column</t>
+  </si>
+  <si>
+    <t>server</t>
+  </si>
+  <si>
+    <t>cable</t>
+  </si>
+  <si>
+    <t>stool</t>
+  </si>
+  <si>
+    <t>cabinet</t>
+  </si>
+  <si>
+    <t>scaffold</t>
+  </si>
+  <si>
+    <t>market stand</t>
+  </si>
+  <si>
+    <t>pillar</t>
+  </si>
+  <si>
+    <t>podium</t>
+  </si>
+  <si>
+    <t>pier</t>
+  </si>
+  <si>
+    <t>crate</t>
+  </si>
+  <si>
+    <t>steering wheel</t>
+  </si>
+  <si>
+    <t>patio</t>
+  </si>
+  <si>
+    <t>curb</t>
+  </si>
+  <si>
+    <t>ramp</t>
+  </si>
+  <si>
+    <t>window ledge</t>
+  </si>
+  <si>
+    <t>shadow</t>
+  </si>
+  <si>
+    <t>parallel</t>
+  </si>
+  <si>
+    <t>lamppost</t>
+  </si>
+  <si>
+    <t>corridor</t>
   </si>
 </sst>
 </file>
@@ -6697,4 +7448,887 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE1BB0A6-53C6-476C-8815-BCA74E0E94A5}">
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="5" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" s="1" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>890</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>891</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>892</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>894</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>895</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>896</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>898</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>899</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>900</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>902</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>903</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>904</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>906</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>907</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>908</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>910</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>911</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>1096</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>914</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>915</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>916</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>918</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>919</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>920</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>1098</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>922</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>923</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>924</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>926</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>927</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>928</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>929</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>1100</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>930</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>931</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>932</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>1101</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>934</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>935</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>936</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>938</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>939</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>940</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>941</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>1103</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>942</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>943</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>944</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>1104</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>946</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>947</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>948</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>949</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>1105</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>950</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>951</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>952</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>1106</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>954</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>955</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>956</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>958</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>959</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>960</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>961</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
+        <v>1108</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>962</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>963</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>964</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>965</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>1109</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>966</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>967</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>968</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>969</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
+        <v>1110</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>970</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>971</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>972</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="7" t="s">
+        <v>1111</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>974</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>975</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>976</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>977</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>978</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>979</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>980</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>981</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="7" t="s">
+        <v>1113</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>982</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>983</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>984</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="7" t="s">
+        <v>1114</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>986</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>987</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>988</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>1115</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>990</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>991</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>992</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>993</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>1116</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>994</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>995</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>996</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>997</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>998</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>999</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>1000</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>1118</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>1004</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="7" t="s">
+        <v>1119</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>1007</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>1008</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="7" t="s">
+        <v>1120</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>1010</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>1011</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>1012</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="7" t="s">
+        <v>1121</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>1014</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>1015</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>1016</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="7" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>1019</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>1020</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>1021</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="7" t="s">
+        <v>1123</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>1023</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>1024</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>1025</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="7" t="s">
+        <v>1124</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>1026</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>1027</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>1028</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>1029</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="7" t="s">
+        <v>1125</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>1030</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>1031</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>1032</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>1033</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="7" t="s">
+        <v>1126</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>1034</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>1035</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>1036</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="7" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>1038</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>1039</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>1040</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7" t="s">
+        <v>1128</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>1042</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>1043</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>1044</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>1045</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="7" t="s">
+        <v>1129</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>1046</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>1049</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="7" t="s">
+        <v>1130</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>1051</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>1052</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="7" t="s">
+        <v>1131</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>1055</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>1056</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="7" t="s">
+        <v>1132</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>1058</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>1059</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>1060</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="7" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>1063</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>1064</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>1065</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="7" t="s">
+        <v>1134</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>1066</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>1067</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>1068</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>1069</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="7" t="s">
+        <v>1135</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>1071</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>1072</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="7" t="s">
+        <v>1136</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>1074</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>1075</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>1076</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>1077</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="7" t="s">
+        <v>1137</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>1078</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>1079</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>1080</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="7" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>1082</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>1083</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>1084</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>1085</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="7" t="s">
+        <v>1139</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>1087</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>1088</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>1089</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
update frontend rate limit and files
</commit_message>
<xml_diff>
--- a/public/flashcard_template.xlsx
+++ b/public/flashcard_template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B87B670-8627-4662-8B7E-21CC9E7DCF29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA86B093-5F2D-4FF6-99C6-540E7166FE6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-23136" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Buổi 2" sheetId="1" r:id="rId1"/>
@@ -15,13 +15,14 @@
     <sheet name="Buổi 6" sheetId="6" r:id="rId5"/>
     <sheet name="Buổi 7" sheetId="7" r:id="rId6"/>
     <sheet name="Buổi 8" sheetId="8" r:id="rId7"/>
+    <sheet name="Voucablry" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1785" uniqueCount="1630">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1848" uniqueCount="1688">
   <si>
     <t>English</t>
   </si>
@@ -4911,6 +4912,180 @@
   </si>
   <si>
     <t>walking stick</t>
+  </si>
+  <si>
+    <t xml:space="preserve">intended </t>
+  </si>
+  <si>
+    <t>dự định</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> motivation </t>
+  </si>
+  <si>
+    <t>động lực</t>
+  </si>
+  <si>
+    <t>improved</t>
+  </si>
+  <si>
+    <t>cải thiện</t>
+  </si>
+  <si>
+    <t xml:space="preserve">appointing </t>
+  </si>
+  <si>
+    <t>bổ nhiệm</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> financed </t>
+  </si>
+  <si>
+    <t>được tài trợ</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> directed </t>
+  </si>
+  <si>
+    <t>được hướng dẫn</t>
+  </si>
+  <si>
+    <t>lời khen ngợi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> compliment</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> promotion </t>
+  </si>
+  <si>
+    <t>khuyến mãi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">encouraged </t>
+  </si>
+  <si>
+    <t>động viên</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> expected </t>
+  </si>
+  <si>
+    <t>hy vọng</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> permitting </t>
+  </si>
+  <si>
+    <t>cho phép</t>
+  </si>
+  <si>
+    <t>evaluate</t>
+  </si>
+  <si>
+    <t>đánh giá</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reliability </t>
+  </si>
+  <si>
+    <t>độ tin cậy</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> inspect </t>
+  </si>
+  <si>
+    <t>thanh tra</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> removal </t>
+  </si>
+  <si>
+    <t>loại bỏ</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> deserved </t>
+  </si>
+  <si>
+    <t>xứng đáng</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> increases </t>
+  </si>
+  <si>
+    <t>tăng lên</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> variety </t>
+  </si>
+  <si>
+    <t>đa dạng</t>
+  </si>
+  <si>
+    <t>proposal</t>
+  </si>
+  <si>
+    <t>sự đề xuất</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> suitable </t>
+  </si>
+  <si>
+    <t>thích hợp</t>
+  </si>
+  <si>
+    <t>extensive</t>
+  </si>
+  <si>
+    <t>rộng rãi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comparable </t>
+  </si>
+  <si>
+    <t>tương đương</t>
+  </si>
+  <si>
+    <t>favorable</t>
+  </si>
+  <si>
+    <t>thuận lợi</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> qualifications </t>
+  </si>
+  <si>
+    <t>trình độ chuyên môn</t>
+  </si>
+  <si>
+    <t>necessary</t>
+  </si>
+  <si>
+    <t>cần thiết</t>
+  </si>
+  <si>
+    <t>become familiar with</t>
+  </si>
+  <si>
+    <t>làm quen với</t>
+  </si>
+  <si>
+    <t>internationally recognized</t>
+  </si>
+  <si>
+    <t>được công nhận quốc tế</t>
+  </si>
+  <si>
+    <t>years of service</t>
+  </si>
+  <si>
+    <t>số năm phục vụ</t>
+  </si>
+  <si>
+    <t>years in operation</t>
+  </si>
+  <si>
+    <t>năm hoạt động</t>
   </si>
 </sst>
 </file>
@@ -11569,4 +11744,499 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A623959F-F63E-46EA-94E2-0B35AAEEBDCC}">
+  <dimension ref="A1:E51"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="5" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>1630</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6" t="s">
+        <v>1631</v>
+      </c>
+      <c r="D2" s="6"/>
+    </row>
+    <row r="3" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>1632</v>
+      </c>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2" t="s">
+        <v>1633</v>
+      </c>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>1634</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2" t="s">
+        <v>1635</v>
+      </c>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
+        <v>1636</v>
+      </c>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>1637</v>
+      </c>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>1638</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>1639</v>
+      </c>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+    </row>
+    <row r="7" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
+        <v>1640</v>
+      </c>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>1641</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+    </row>
+    <row r="8" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>1643</v>
+      </c>
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
+        <v>1642</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+    </row>
+    <row r="9" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="7" t="s">
+        <v>1644</v>
+      </c>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>1645</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="7" t="s">
+        <v>1646</v>
+      </c>
+      <c r="B10" s="2"/>
+      <c r="C10" s="2" t="s">
+        <v>1647</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7" t="s">
+        <v>1648</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2" t="s">
+        <v>1649</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="7" t="s">
+        <v>1650</v>
+      </c>
+      <c r="B12" s="2"/>
+      <c r="C12" s="2" t="s">
+        <v>1651</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+    </row>
+    <row r="13" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>1652</v>
+      </c>
+      <c r="B13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>1653</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>1654</v>
+      </c>
+      <c r="B14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>1655</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+    </row>
+    <row r="15" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>1656</v>
+      </c>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>1657</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>1658</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>1659</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+    </row>
+    <row r="17" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>1660</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2" t="s">
+        <v>1661</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>1662</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2" t="s">
+        <v>1663</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
+        <v>1664</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2" t="s">
+        <v>1665</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="7" t="s">
+        <v>1666</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2" t="s">
+        <v>1667</v>
+      </c>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+    </row>
+    <row r="21" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="7" t="s">
+        <v>1668</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>1669</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="7" t="s">
+        <v>1670</v>
+      </c>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2" t="s">
+        <v>1671</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="7" t="s">
+        <v>1672</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2" t="s">
+        <v>1673</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+    </row>
+    <row r="24" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="7" t="s">
+        <v>1674</v>
+      </c>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2" t="s">
+        <v>1675</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+    </row>
+    <row r="25" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="7" t="s">
+        <v>1676</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2" t="s">
+        <v>1677</v>
+      </c>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+    </row>
+    <row r="26" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="7" t="s">
+        <v>1678</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2" t="s">
+        <v>1679</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+    </row>
+    <row r="27" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="7" t="s">
+        <v>1680</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2" t="s">
+        <v>1681</v>
+      </c>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+    </row>
+    <row r="28" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="7" t="s">
+        <v>1682</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2" t="s">
+        <v>1683</v>
+      </c>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+    </row>
+    <row r="29" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="7" t="s">
+        <v>1684</v>
+      </c>
+      <c r="B29" s="2"/>
+      <c r="C29" s="2" t="s">
+        <v>1685</v>
+      </c>
+      <c r="D29" s="2"/>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" ht="33.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="7" t="s">
+        <v>1686</v>
+      </c>
+      <c r="B30" s="2"/>
+      <c r="C30" s="2" t="s">
+        <v>1687</v>
+      </c>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+    </row>
+    <row r="31" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="7"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+    </row>
+    <row r="32" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="7"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+    </row>
+    <row r="33" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="7"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+    </row>
+    <row r="34" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="7"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+    </row>
+    <row r="35" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="7"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+    </row>
+    <row r="36" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="7"/>
+      <c r="B36" s="2"/>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="7"/>
+      <c r="B37" s="2"/>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+    </row>
+    <row r="38" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="7"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+    </row>
+    <row r="39" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="7"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="7"/>
+      <c r="B40" s="2"/>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+    </row>
+    <row r="41" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="7"/>
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+    </row>
+    <row r="42" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="7"/>
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+    </row>
+    <row r="43" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="7"/>
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+    </row>
+    <row r="44" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="7"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+    </row>
+    <row r="45" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="7"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="7"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+    </row>
+    <row r="47" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="7"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+    </row>
+    <row r="48" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="7"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+    </row>
+    <row r="49" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="7"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+    </row>
+    <row r="50" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="7"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+    </row>
+    <row r="51" spans="1:5" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="7"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>